<commit_message>
Copyright polish: full originals in Excel and weekly cards, accurate wording
From the final review: the Excel By theme rows of translated headlines are
tall enough for the original, the weekly index card shows the original under
a translated lead headline, the Method page and README say summaries and
abstracts are no longer saved (rather than never kept), and the primary
source is held to 120 characters with its ellipsis.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2cbJQGUUZpwz34g4NBxNT
</commit_message>
<xml_diff>
--- a/docs/exports/2026-Q4.xlsx
+++ b/docs/exports/2026-Q4.xlsx
@@ -17434,7 +17434,7 @@
         </is>
       </c>
     </row>
-    <row r="26" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="26" outlineLevel="1" ht="104" customHeight="1">
       <c r="A26" s="190" t="n">
         <v>57</v>
       </c>
@@ -17925,7 +17925,7 @@
         </is>
       </c>
     </row>
-    <row r="38" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="38" outlineLevel="1" ht="79" customHeight="1">
       <c r="A38" s="190" t="n">
         <v>70</v>
       </c>
@@ -18048,7 +18048,7 @@
         </is>
       </c>
     </row>
-    <row r="41" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="41" outlineLevel="1" ht="79" customHeight="1">
       <c r="A41" s="190" t="n">
         <v>17</v>
       </c>
@@ -18599,7 +18599,7 @@
         </is>
       </c>
     </row>
-    <row r="56" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="56" outlineLevel="1" ht="79" customHeight="1">
       <c r="A56" s="190" t="n">
         <v>51</v>
       </c>
@@ -18785,7 +18785,7 @@
         </is>
       </c>
     </row>
-    <row r="62" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="62" outlineLevel="1" ht="79" customHeight="1">
       <c r="A62" s="190" t="n">
         <v>74</v>
       </c>
@@ -19030,7 +19030,7 @@
         </is>
       </c>
     </row>
-    <row r="68" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="68" outlineLevel="1" ht="91.5" customHeight="1">
       <c r="A68" s="190" t="n">
         <v>83</v>
       </c>
@@ -19846,7 +19846,7 @@
         </is>
       </c>
     </row>
-    <row r="88" outlineLevel="1" ht="66.5" customHeight="1">
+    <row r="88" outlineLevel="1" ht="91.5" customHeight="1">
       <c r="A88" s="190" t="n">
         <v>44</v>
       </c>

</xml_diff>